<commit_message>
docs: liens des issues et corrections du rapport de tests
</commit_message>
<xml_diff>
--- a/docs/Plan_de_tests_Lot1_Resultats__.xlsx
+++ b/docs/Plan_de_tests_Lot1_Resultats__.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="251">
   <si>
     <t>Plan de tests – Lot 1 – Projet Skull M1S1</t>
   </si>
@@ -799,6 +799,17 @@
     <t>PlayerService / Maxime</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="20"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://github.com/Rayanxdn/Skull_Game_M1S1/issues/14</t>
+    </r>
+  </si>
+  <si>
     <t>Ouvert</t>
   </si>
   <si>
@@ -814,16 +825,49 @@
     <t>PlayerService (sécurité, à confirmer)</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="20"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://github.com/Rayanxdn/Skull_Game_M1S1/issues/15</t>
+    </r>
+  </si>
+  <si>
     <t>A03</t>
   </si>
   <si>
     <t>Même comportement de T20 sur PUT /players/{id}/ban avec un token joueur valide.même comportement que A02</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="20"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://github.com/Rayanxdn/Skull_Game_M1S1/issues/16</t>
+    </r>
+  </si>
+  <si>
     <t>A04</t>
   </si>
   <si>
     <t>Un joueur banni utilisant un token valide reçoit 401 au lieu de 403.même comportement que A02</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="20"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>https://github.com/Rayanxdn/Skull_Game_M1S1/issues/18</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -834,7 +878,7 @@
     <numFmt numFmtId="0" formatCode="General"/>
     <numFmt numFmtId="59" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -846,12 +890,7 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14"/>
+      <sz val="15"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
@@ -892,7 +931,7 @@
     </font>
     <font>
       <sz val="8"/>
-      <color indexed="18"/>
+      <color indexed="17"/>
       <name val="Courier"/>
     </font>
     <font>
@@ -911,11 +950,6 @@
       <name val="Times Roman"/>
     </font>
     <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color indexed="8"/>
       <name val="Arial"/>
@@ -932,7 +966,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="19"/>
+      <color indexed="18"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -942,8 +976,14 @@
     </font>
     <font>
       <sz val="10"/>
+      <color indexed="19"/>
+      <name val="Courier"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
       <color indexed="20"/>
-      <name val="Courier"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1061,38 +1101,41 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="59" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="5" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1104,98 +1147,83 @@
     <xf numFmtId="49" fontId="9" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="14" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="15" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="1" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="16" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="9" fontId="16" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="20" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="1" fontId="18" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1209,14 +1237,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="14"/>
           <bgColor indexed="16"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="14"/>
-          <bgColor indexed="17"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1240,11 +1260,11 @@
       <rgbColor rgb="fffff2cc"/>
       <rgbColor rgb="00000000"/>
       <rgbColor rgb="ffc6efce"/>
-      <rgbColor rgb="ffffc7ce"/>
       <rgbColor rgb="ffffeb9c"/>
       <rgbColor rgb="ff020202"/>
       <rgbColor rgb="ff808080"/>
       <rgbColor rgb="ff050505"/>
+      <rgbColor rgb="ff0000ff"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1443,9 +1463,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1477,10 +1500,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1719,9 +1742,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -2025,10 +2051,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -3688,9 +3714,6 @@
       <formula>"OK"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal" stopIfTrue="1">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal" stopIfTrue="1">
       <formula>"Bloqué"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3722,262 +3745,262 @@
       <c r="A1" t="s" s="21">
         <v>218</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="23"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" ht="14.6" customHeight="1">
-      <c r="A3" t="s" s="25">
+      <c r="A3" t="s" s="22">
         <v>9</v>
       </c>
-      <c r="B3" t="s" s="25">
+      <c r="B3" t="s" s="22">
         <v>219</v>
       </c>
-      <c r="C3" t="s" s="25">
+      <c r="C3" t="s" s="22">
         <v>220</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="14.6" customHeight="1">
-      <c r="A4" t="s" s="27">
+      <c r="A4" t="s" s="24">
         <v>19</v>
       </c>
-      <c r="B4" s="28" cm="1">
+      <c r="B4" s="25" cm="1">
         <f t="array" ref="B4">COUNTIF('Plan de tests Lot 1'!$I$4:$I$38,A4)</f>
         <v>32</v>
       </c>
-      <c r="C4" s="29" cm="1">
+      <c r="C4" s="26" cm="1">
         <f t="array" ref="C4">_xlfn.IFERROR(B4/$B$8,0)</f>
         <v>0.914285714285714</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="14.6" customHeight="1">
-      <c r="A5" t="s" s="27">
+      <c r="A5" t="s" s="24">
         <v>128</v>
       </c>
-      <c r="B5" s="28" cm="1">
+      <c r="B5" s="25" cm="1">
         <f t="array" ref="B5">COUNTIF('Plan de tests Lot 1'!$I$4:$I$38,A5)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="29" cm="1">
+      <c r="C5" s="26" cm="1">
         <f t="array" ref="C5">_xlfn.IFERROR(B5/$B$8,0)</f>
         <v>0.0857142857142857</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" ht="14.6" customHeight="1">
-      <c r="A6" t="s" s="27">
+      <c r="A6" t="s" s="24">
         <v>221</v>
       </c>
-      <c r="B6" s="28" cm="1">
+      <c r="B6" s="25" cm="1">
         <f t="array" ref="B6">COUNTIF('Plan de tests Lot 1'!$I$4:$I$38,A6)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="29" cm="1">
+      <c r="C6" s="26" cm="1">
         <f t="array" ref="C6">_xlfn.IFERROR(B6/$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" ht="14.6" customHeight="1">
-      <c r="A7" t="s" s="27">
+      <c r="A7" t="s" s="24">
         <v>222</v>
       </c>
-      <c r="B7" s="28" cm="1">
+      <c r="B7" s="25" cm="1">
         <f t="array" ref="B7">COUNTIF('Plan de tests Lot 1'!$I$4:$I$38,A7)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="29" cm="1">
+      <c r="C7" s="26" cm="1">
         <f t="array" ref="C7">_xlfn.IFERROR(B7/$B$8,0)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" ht="14.6" customHeight="1">
-      <c r="A8" t="s" s="27">
+      <c r="A8" t="s" s="24">
         <v>223</v>
       </c>
-      <c r="B8" s="28" cm="1">
+      <c r="B8" s="25" cm="1">
         <f t="array" ref="B8">SUM(B4:B7)</f>
         <v>35</v>
       </c>
-      <c r="C8" s="29" cm="1">
+      <c r="C8" s="26" cm="1">
         <f t="array" ref="C8">SUM(C4:C7)</f>
         <v>1</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" ht="14.6" customHeight="1">
-      <c r="A10" t="s" s="31">
+      <c r="A10" t="s" s="28">
         <v>224</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="23"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" ht="14.6" customHeight="1">
-      <c r="A11" t="s" s="25">
+      <c r="A11" t="s" s="22">
         <v>2</v>
       </c>
-      <c r="B11" t="s" s="25">
+      <c r="B11" t="s" s="22">
         <v>223</v>
       </c>
-      <c r="C11" t="s" s="25">
+      <c r="C11" t="s" s="22">
         <v>19</v>
       </c>
-      <c r="D11" t="s" s="25">
+      <c r="D11" t="s" s="22">
         <v>128</v>
       </c>
-      <c r="E11" s="32"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" ht="14.6" customHeight="1">
-      <c r="A12" t="s" s="27">
+      <c r="A12" t="s" s="24">
         <v>14</v>
       </c>
-      <c r="B12" s="28" cm="1">
+      <c r="B12" s="25" cm="1">
         <f t="array" ref="B12">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A12)</f>
         <v>5</v>
       </c>
-      <c r="C12" s="28" cm="1">
+      <c r="C12" s="25" cm="1">
         <f t="array" ref="C12">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A12,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>5</v>
       </c>
-      <c r="D12" s="28" cm="1">
+      <c r="D12" s="25" cm="1">
         <f t="array" ref="D12">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A12,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="32"/>
+      <c r="E12" s="23"/>
     </row>
     <row r="13" ht="14.6" customHeight="1">
-      <c r="A13" t="s" s="27">
+      <c r="A13" t="s" s="24">
         <v>45</v>
       </c>
-      <c r="B13" s="28" cm="1">
+      <c r="B13" s="25" cm="1">
         <f t="array" ref="B13">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A13)</f>
         <v>4</v>
       </c>
-      <c r="C13" s="28" cm="1">
+      <c r="C13" s="25" cm="1">
         <f t="array" ref="C13">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A13,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>4</v>
       </c>
-      <c r="D13" s="28" cm="1">
+      <c r="D13" s="25" cm="1">
         <f t="array" ref="D13">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A13,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>0</v>
       </c>
-      <c r="E13" s="32"/>
+      <c r="E13" s="23"/>
     </row>
     <row r="14" ht="14.6" customHeight="1">
-      <c r="A14" t="s" s="27">
+      <c r="A14" t="s" s="24">
         <v>67</v>
       </c>
-      <c r="B14" s="28" cm="1">
+      <c r="B14" s="25" cm="1">
         <f t="array" ref="B14">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A14)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="28" cm="1">
+      <c r="C14" s="25" cm="1">
         <f t="array" ref="C14">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A14,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>5</v>
       </c>
-      <c r="D14" s="28" cm="1">
+      <c r="D14" s="25" cm="1">
         <f t="array" ref="D14">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A14,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>0</v>
       </c>
-      <c r="E14" s="32"/>
+      <c r="E14" s="23"/>
     </row>
     <row r="15" ht="14.6" customHeight="1">
-      <c r="A15" t="s" s="27">
+      <c r="A15" t="s" s="24">
         <v>95</v>
       </c>
-      <c r="B15" s="28" cm="1">
+      <c r="B15" s="25" cm="1">
         <f t="array" ref="B15">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A15)</f>
         <v>9</v>
       </c>
-      <c r="C15" s="28" cm="1">
+      <c r="C15" s="25" cm="1">
         <f t="array" ref="C15">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A15,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>8</v>
       </c>
-      <c r="D15" s="28" cm="1">
+      <c r="D15" s="25" cm="1">
         <f t="array" ref="D15">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A15,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>1</v>
       </c>
-      <c r="E15" s="32"/>
+      <c r="E15" s="23"/>
     </row>
     <row r="16" ht="14.6" customHeight="1">
-      <c r="A16" t="s" s="27">
+      <c r="A16" t="s" s="24">
         <v>149</v>
       </c>
-      <c r="B16" s="28" cm="1">
+      <c r="B16" s="25" cm="1">
         <f t="array" ref="B16">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A16)</f>
         <v>2</v>
       </c>
-      <c r="C16" s="28" cm="1">
+      <c r="C16" s="25" cm="1">
         <f t="array" ref="C16">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A16,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>2</v>
       </c>
-      <c r="D16" s="28" cm="1">
+      <c r="D16" s="25" cm="1">
         <f t="array" ref="D16">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A16,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>0</v>
       </c>
-      <c r="E16" s="32"/>
+      <c r="E16" s="23"/>
     </row>
     <row r="17" ht="14.6" customHeight="1">
-      <c r="A17" t="s" s="27">
+      <c r="A17" t="s" s="24">
         <v>162</v>
       </c>
-      <c r="B17" s="28" cm="1">
+      <c r="B17" s="25" cm="1">
         <f t="array" ref="B17">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A17)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="28" cm="1">
+      <c r="C17" s="25" cm="1">
         <f t="array" ref="C17">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A17,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>6</v>
       </c>
-      <c r="D17" s="28" cm="1">
+      <c r="D17" s="25" cm="1">
         <f t="array" ref="D17">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A17,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>2</v>
       </c>
-      <c r="E17" s="32"/>
+      <c r="E17" s="23"/>
     </row>
     <row r="18" ht="14.6" customHeight="1">
-      <c r="A18" t="s" s="27">
+      <c r="A18" t="s" s="24">
         <v>207</v>
       </c>
-      <c r="B18" s="28" cm="1">
+      <c r="B18" s="25" cm="1">
         <f t="array" ref="B18">COUNTIF('Plan de tests Lot 1'!$B$4:$B$38,A18)</f>
         <v>2</v>
       </c>
-      <c r="C18" s="28" cm="1">
+      <c r="C18" s="25" cm="1">
         <f t="array" ref="C18">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A18,'Plan de tests Lot 1'!$I$4:$I$38,"OK")</f>
         <v>2</v>
       </c>
-      <c r="D18" s="28" cm="1">
+      <c r="D18" s="25" cm="1">
         <f t="array" ref="D18">_xlfn.COUNTIFS('Plan de tests Lot 1'!$B$4:$B$38,A18,'Plan de tests Lot 1'!$I$4:$I$38,"KO")</f>
         <v>0</v>
       </c>
-      <c r="E18" s="32"/>
+      <c r="E18" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
@@ -3993,431 +4016,439 @@
   <dimension ref="A1:I31"/>
   <sheetFormatPr defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="7" style="33" customWidth="1"/>
-    <col min="2" max="2" width="14" style="33" customWidth="1"/>
-    <col min="3" max="3" width="50" style="33" customWidth="1"/>
-    <col min="4" max="4" width="12" style="33" customWidth="1"/>
-    <col min="5" max="5" width="24" style="33" customWidth="1"/>
-    <col min="6" max="6" width="36" style="33" customWidth="1"/>
-    <col min="7" max="7" width="12" style="33" customWidth="1"/>
-    <col min="8" max="9" width="14" style="33" customWidth="1"/>
-    <col min="10" max="16384" width="8.67188" style="33" customWidth="1"/>
+    <col min="1" max="1" width="7" style="29" customWidth="1"/>
+    <col min="2" max="2" width="14" style="29" customWidth="1"/>
+    <col min="3" max="3" width="50" style="29" customWidth="1"/>
+    <col min="4" max="4" width="12" style="29" customWidth="1"/>
+    <col min="5" max="5" width="24" style="29" customWidth="1"/>
+    <col min="6" max="6" width="36" style="29" customWidth="1"/>
+    <col min="7" max="7" width="12" style="29" customWidth="1"/>
+    <col min="8" max="9" width="14" style="29" customWidth="1"/>
+    <col min="10" max="16384" width="8.67188" style="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.6" customHeight="1">
-      <c r="A1" t="s" s="25">
+      <c r="A1" t="s" s="22">
         <v>225</v>
       </c>
-      <c r="B1" t="s" s="25">
+      <c r="B1" t="s" s="22">
         <v>226</v>
       </c>
-      <c r="C1" t="s" s="25">
+      <c r="C1" t="s" s="22">
         <v>227</v>
       </c>
-      <c r="D1" t="s" s="25">
+      <c r="D1" t="s" s="22">
         <v>228</v>
       </c>
-      <c r="E1" t="s" s="25">
+      <c r="E1" t="s" s="22">
         <v>229</v>
       </c>
-      <c r="F1" t="s" s="25">
+      <c r="F1" t="s" s="22">
         <v>230</v>
       </c>
-      <c r="G1" t="s" s="25">
+      <c r="G1" t="s" s="22">
         <v>9</v>
       </c>
-      <c r="H1" t="s" s="25">
+      <c r="H1" t="s" s="22">
         <v>231</v>
       </c>
-      <c r="I1" t="s" s="25">
+      <c r="I1" t="s" s="22">
         <v>232</v>
       </c>
     </row>
     <row r="2" ht="13.65" customHeight="1">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" ht="27" customHeight="1">
-      <c r="A3" t="s" s="35">
+      <c r="A3" t="s" s="31">
         <v>233</v>
       </c>
-      <c r="B3" t="s" s="35">
+      <c r="B3" t="s" s="31">
         <v>234</v>
       </c>
-      <c r="C3" t="s" s="36">
+      <c r="C3" t="s" s="32">
         <v>235</v>
       </c>
-      <c r="D3" t="s" s="37">
+      <c r="D3" t="s" s="33">
         <v>236</v>
       </c>
-      <c r="E3" t="s" s="35">
+      <c r="E3" t="s" s="31">
         <v>237</v>
       </c>
-      <c r="F3" s="38"/>
-      <c r="G3" t="s" s="35">
+      <c r="F3" t="s" s="31">
         <v>238</v>
       </c>
-      <c r="H3" s="39">
+      <c r="G3" t="s" s="31">
+        <v>239</v>
+      </c>
+      <c r="H3" s="34">
         <v>46321</v>
       </c>
-      <c r="I3" s="40"/>
+      <c r="I3" s="35"/>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" t="s" s="35">
+      <c r="A4" t="s" s="31">
+        <v>240</v>
+      </c>
+      <c r="B4" t="s" s="31">
+        <v>123</v>
+      </c>
+      <c r="C4" t="s" s="36">
+        <v>241</v>
+      </c>
+      <c r="D4" t="s" s="31">
+        <v>242</v>
+      </c>
+      <c r="E4" t="s" s="37">
+        <v>243</v>
+      </c>
+      <c r="F4" t="s" s="31">
+        <v>244</v>
+      </c>
+      <c r="G4" t="s" s="31">
         <v>239</v>
       </c>
-      <c r="B4" t="s" s="35">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s" s="41">
-        <v>240</v>
-      </c>
-      <c r="D4" t="s" s="35">
-        <v>241</v>
-      </c>
-      <c r="E4" t="s" s="42">
+      <c r="H4" s="34">
+        <v>46321</v>
+      </c>
+      <c r="I4" s="35"/>
+    </row>
+    <row r="5" ht="27" customHeight="1">
+      <c r="A5" t="s" s="31">
+        <v>245</v>
+      </c>
+      <c r="B5" t="s" s="31">
+        <v>168</v>
+      </c>
+      <c r="C5" t="s" s="31">
+        <v>246</v>
+      </c>
+      <c r="D5" t="s" s="31">
         <v>242</v>
       </c>
-      <c r="F4" s="40"/>
-      <c r="G4" t="s" s="35">
-        <v>238</v>
-      </c>
-      <c r="H4" s="39">
+      <c r="E5" t="s" s="37">
+        <v>243</v>
+      </c>
+      <c r="F5" t="s" s="31">
+        <v>247</v>
+      </c>
+      <c r="G5" t="s" s="31">
+        <v>239</v>
+      </c>
+      <c r="H5" s="34">
         <v>46321</v>
       </c>
-      <c r="I4" s="40"/>
-    </row>
-    <row r="5" ht="27" customHeight="1">
-      <c r="A5" t="s" s="35">
+      <c r="I5" s="35"/>
+    </row>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" t="s" s="31">
+        <v>248</v>
+      </c>
+      <c r="B6" t="s" s="31">
+        <v>184</v>
+      </c>
+      <c r="C6" t="s" s="31">
+        <v>249</v>
+      </c>
+      <c r="D6" t="s" s="31">
+        <v>242</v>
+      </c>
+      <c r="E6" t="s" s="37">
         <v>243</v>
       </c>
-      <c r="B5" t="s" s="35">
-        <v>168</v>
-      </c>
-      <c r="C5" t="s" s="35">
-        <v>244</v>
-      </c>
-      <c r="D5" t="s" s="35">
-        <v>241</v>
-      </c>
-      <c r="E5" t="s" s="42">
-        <v>242</v>
-      </c>
-      <c r="F5" s="40"/>
-      <c r="G5" t="s" s="35">
-        <v>238</v>
-      </c>
-      <c r="H5" s="39">
+      <c r="F6" t="s" s="31">
+        <v>250</v>
+      </c>
+      <c r="G6" t="s" s="31">
+        <v>239</v>
+      </c>
+      <c r="H6" s="34">
         <v>46321</v>
       </c>
-      <c r="I5" s="40"/>
-    </row>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" t="s" s="35">
-        <v>245</v>
-      </c>
-      <c r="B6" t="s" s="35">
-        <v>184</v>
-      </c>
-      <c r="C6" t="s" s="35">
-        <v>246</v>
-      </c>
-      <c r="D6" t="s" s="35">
-        <v>241</v>
-      </c>
-      <c r="E6" t="s" s="42">
-        <v>242</v>
-      </c>
-      <c r="F6" s="40"/>
-      <c r="G6" t="s" s="35">
-        <v>238</v>
-      </c>
-      <c r="H6" s="39">
-        <v>46321</v>
-      </c>
-      <c r="I6" s="40"/>
+      <c r="I6" s="35"/>
     </row>
     <row r="7" ht="13.65" customHeight="1">
-      <c r="A7" s="40"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="38"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
       <c r="G7" s="38"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="40"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" ht="13.65" customHeight="1">
-      <c r="A8" s="40"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="A8" s="35"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="38"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
       <c r="G8" s="38"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
     </row>
     <row r="9" ht="13.65" customHeight="1">
-      <c r="A9" s="40"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="38"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
       <c r="G9" s="38"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="40"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
     </row>
     <row r="10" ht="13.65" customHeight="1">
-      <c r="A10" s="40"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="38"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
       <c r="G10" s="38"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
     </row>
     <row r="11" ht="13.65" customHeight="1">
-      <c r="A11" s="40"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
       <c r="D11" s="38"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
       <c r="G11" s="38"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
-      <c r="A12" s="40"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
       <c r="D12" s="38"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
       <c r="G12" s="38"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
     </row>
     <row r="13" ht="13.65" customHeight="1">
-      <c r="A13" s="40"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
+      <c r="A13" s="35"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
       <c r="D13" s="38"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
       <c r="G13" s="38"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
     </row>
     <row r="14" ht="13.65" customHeight="1">
-      <c r="A14" s="40"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
       <c r="D14" s="38"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
       <c r="G14" s="38"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
     </row>
     <row r="15" ht="13.65" customHeight="1">
-      <c r="A15" s="40"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
       <c r="D15" s="38"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
       <c r="G15" s="38"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
     </row>
     <row r="16" ht="13.65" customHeight="1">
-      <c r="A16" s="40"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
       <c r="D16" s="38"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
       <c r="G16" s="38"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
     </row>
     <row r="17" ht="13.65" customHeight="1">
-      <c r="A17" s="40"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
       <c r="D17" s="38"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
       <c r="G17" s="38"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
     </row>
     <row r="18" ht="13.65" customHeight="1">
-      <c r="A18" s="40"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
       <c r="D18" s="38"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
       <c r="G18" s="38"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
     </row>
     <row r="19" ht="13.65" customHeight="1">
-      <c r="A19" s="40"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
+      <c r="A19" s="35"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
       <c r="D19" s="38"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
       <c r="G19" s="38"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
     </row>
     <row r="20" ht="13.65" customHeight="1">
-      <c r="A20" s="40"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
       <c r="D20" s="38"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
       <c r="G20" s="38"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
     </row>
     <row r="21" ht="13.65" customHeight="1">
-      <c r="A21" s="40"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
+      <c r="A21" s="35"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
       <c r="D21" s="38"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
       <c r="G21" s="38"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
     </row>
     <row r="22" ht="13.65" customHeight="1">
-      <c r="A22" s="40"/>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
+      <c r="A22" s="35"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
       <c r="D22" s="38"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
       <c r="G22" s="38"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
     </row>
     <row r="23" ht="13.65" customHeight="1">
-      <c r="A23" s="40"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
+      <c r="A23" s="35"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
       <c r="D23" s="38"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
       <c r="G23" s="38"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
     </row>
     <row r="24" ht="13.65" customHeight="1">
-      <c r="A24" s="40"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
+      <c r="A24" s="35"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
       <c r="D24" s="38"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
       <c r="G24" s="38"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
     </row>
     <row r="25" ht="13.65" customHeight="1">
-      <c r="A25" s="40"/>
-      <c r="B25" s="40"/>
-      <c r="C25" s="40"/>
+      <c r="A25" s="35"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
       <c r="D25" s="38"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
       <c r="G25" s="38"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
     </row>
     <row r="26" ht="13.65" customHeight="1">
-      <c r="A26" s="40"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
+      <c r="A26" s="35"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="35"/>
       <c r="D26" s="38"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
       <c r="G26" s="38"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="40"/>
+      <c r="H26" s="35"/>
+      <c r="I26" s="35"/>
     </row>
     <row r="27" ht="13.65" customHeight="1">
-      <c r="A27" s="40"/>
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
+      <c r="A27" s="35"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
       <c r="D27" s="38"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
       <c r="G27" s="38"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="35"/>
     </row>
     <row r="28" ht="13.65" customHeight="1">
-      <c r="A28" s="40"/>
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
       <c r="D28" s="38"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
       <c r="G28" s="38"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
     </row>
     <row r="29" ht="13.65" customHeight="1">
-      <c r="A29" s="40"/>
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="35"/>
       <c r="D29" s="38"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
       <c r="G29" s="38"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
     </row>
     <row r="30" ht="13.65" customHeight="1">
-      <c r="A30" s="40"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="40"/>
+      <c r="A30" s="35"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
       <c r="G30" s="38"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
     </row>
     <row r="31" ht="13.65" customHeight="1">
-      <c r="A31" s="40"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
+      <c r="A31" s="35"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
       <c r="D31" s="38"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
       <c r="G31" s="38"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4428,6 +4459,12 @@
       <formula1>"Ouvert,En cours,Corrigé,Retesté OK"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="F3" r:id="rId1" location="" tooltip="" display="https://github.com/Rayanxdn/Skull_Game_M1S1/issues/14"/>
+    <hyperlink ref="F4" r:id="rId2" location="" tooltip="" display="https://github.com/Rayanxdn/Skull_Game_M1S1/issues/15"/>
+    <hyperlink ref="F5" r:id="rId3" location="" tooltip="" display="https://github.com/Rayanxdn/Skull_Game_M1S1/issues/16"/>
+    <hyperlink ref="F6" r:id="rId4" location="" tooltip="" display="https://github.com/Rayanxdn/Skull_Game_M1S1/issues/18"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>

</xml_diff>